<commit_message>
Protocolo Cautelar: oferta, métricas, criativos, mockup e pacotes de entrega
- Oferta com bumps reais, economia da venda, CPA/ROAS e plano de teste
- Mockup 3D e 12 criativos PNG (4 conceitos x 3 formatos)
- Guia 'Comece por aqui' e ZIPs do kit principal e dos dois bumps
- Faixa < 0,7x (peça mais fina) no app e na planilha de pintura
- Correção: negrito após títulos com atributos e itens de checklist
- Checklist de qualidade com pendências normativas

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013g5H3uXTK57K7CqufyRZ9d
</commit_message>
<xml_diff>
--- a/ebooks/protocolo-cautelar/03-materiais/planilhas/02-mapa-de-pintura.xlsx
+++ b/ebooks/protocolo-cautelar/03-materiais/planilhas/02-mapa-de-pintura.xlsx
@@ -13,7 +13,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Capa'!$A$1:$F$30</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Mapa'!$9:$9</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Mapa'!$A$1:$L$38</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Mapa'!$A$1:$L$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -341,7 +341,20 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="004F7FB0"/>
+          <bgColor rgb="004F7FB0"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <name val="Calibri"/>
@@ -406,6 +419,13 @@
         <name val="Calibri"/>
         <b val="1"/>
         <color rgb="00B87F00"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="004F7FB0"/>
       </font>
     </dxf>
   </dxfs>
@@ -953,11 +973,11 @@
       </c>
       <c r="F16" s="6" t="n"/>
     </row>
-    <row r="17" ht="32" customHeight="1">
+    <row r="17" ht="46" customHeight="1">
       <c r="A17" s="6" t="n"/>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>3. Razão = média da peça ÷ referência. O status e a cor mudam sozinhos conforme os limites da aba (editáveis).</t>
+          <t>3. Razão = média da peça ÷ referência. O status e a cor mudam sozinhos conforme os limites da aba (editáveis): &lt;0,7 mais fina (investigar); ≤1,3 compatível; ≤2 provável repintura; &gt;2 com massa/reparo.</t>
         </is>
       </c>
       <c r="F17" s="6" t="n"/>
@@ -1203,7 +1223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1350,6 +1370,23 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>Limite mais fina (razão &lt;)</t>
+        </is>
+      </c>
+      <c r="F8" s="22" t="n"/>
+      <c r="G8" s="20" t="n"/>
+      <c r="H8" s="23" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>abaixo disso: mais fina — investigar (polimento ou peça substituída)</t>
+        </is>
+      </c>
+    </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="27" t="inlineStr">
         <is>
@@ -1451,7 +1488,7 @@
         <v/>
       </c>
       <c r="K10" s="26">
-        <f>IF(B10="Plástico","NÃO MEDIR (plástico)",IF(I10="","— sem leitura",IF(I10&lt;=$H$5,"Compatível",IF(I10&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo"))))</f>
+        <f>IF(B10="Plástico","NÃO MEDIR (plástico)",IF(I10="","— sem leitura",IF(I10&lt;$H$8,"Mais fina: investigar (polimento ou peça substituída)",IF(I10&lt;=$H$5,"Compatível",IF(I10&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo")))))</f>
         <v/>
       </c>
       <c r="L10" s="11" t="n"/>
@@ -1495,7 +1532,7 @@
         <v/>
       </c>
       <c r="K11" s="26">
-        <f>IF(B11="Plástico","NÃO MEDIR (plástico)",IF(I11="","— sem leitura",IF(I11&lt;=$H$5,"Compatível",IF(I11&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo"))))</f>
+        <f>IF(B11="Plástico","NÃO MEDIR (plástico)",IF(I11="","— sem leitura",IF(I11&lt;$H$8,"Mais fina: investigar (polimento ou peça substituída)",IF(I11&lt;=$H$5,"Compatível",IF(I11&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo")))))</f>
         <v/>
       </c>
       <c r="L11" s="11" t="n"/>
@@ -1539,7 +1576,7 @@
         <v/>
       </c>
       <c r="K12" s="26">
-        <f>IF(B12="Plástico","NÃO MEDIR (plástico)",IF(I12="","— sem leitura",IF(I12&lt;=$H$5,"Compatível",IF(I12&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo"))))</f>
+        <f>IF(B12="Plástico","NÃO MEDIR (plástico)",IF(I12="","— sem leitura",IF(I12&lt;$H$8,"Mais fina: investigar (polimento ou peça substituída)",IF(I12&lt;=$H$5,"Compatível",IF(I12&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo")))))</f>
         <v/>
       </c>
       <c r="L12" s="11" t="n"/>
@@ -1583,7 +1620,7 @@
         <v/>
       </c>
       <c r="K13" s="26">
-        <f>IF(B13="Plástico","NÃO MEDIR (plástico)",IF(I13="","— sem leitura",IF(I13&lt;=$H$5,"Compatível",IF(I13&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo"))))</f>
+        <f>IF(B13="Plástico","NÃO MEDIR (plástico)",IF(I13="","— sem leitura",IF(I13&lt;$H$8,"Mais fina: investigar (polimento ou peça substituída)",IF(I13&lt;=$H$5,"Compatível",IF(I13&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo")))))</f>
         <v/>
       </c>
       <c r="L13" s="11" t="n"/>
@@ -1627,7 +1664,7 @@
         <v/>
       </c>
       <c r="K14" s="26">
-        <f>IF(B14="Plástico","NÃO MEDIR (plástico)",IF(I14="","— sem leitura",IF(I14&lt;=$H$5,"Compatível",IF(I14&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo"))))</f>
+        <f>IF(B14="Plástico","NÃO MEDIR (plástico)",IF(I14="","— sem leitura",IF(I14&lt;$H$8,"Mais fina: investigar (polimento ou peça substituída)",IF(I14&lt;=$H$5,"Compatível",IF(I14&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo")))))</f>
         <v/>
       </c>
       <c r="L14" s="11" t="n"/>
@@ -1671,7 +1708,7 @@
         <v/>
       </c>
       <c r="K15" s="26">
-        <f>IF(B15="Plástico","NÃO MEDIR (plástico)",IF(I15="","— sem leitura",IF(I15&lt;=$H$5,"Compatível",IF(I15&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo"))))</f>
+        <f>IF(B15="Plástico","NÃO MEDIR (plástico)",IF(I15="","— sem leitura",IF(I15&lt;$H$8,"Mais fina: investigar (polimento ou peça substituída)",IF(I15&lt;=$H$5,"Compatível",IF(I15&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo")))))</f>
         <v/>
       </c>
       <c r="L15" s="11" t="n"/>
@@ -1715,7 +1752,7 @@
         <v/>
       </c>
       <c r="K16" s="26">
-        <f>IF(B16="Plástico","NÃO MEDIR (plástico)",IF(I16="","— sem leitura",IF(I16&lt;=$H$5,"Compatível",IF(I16&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo"))))</f>
+        <f>IF(B16="Plástico","NÃO MEDIR (plástico)",IF(I16="","— sem leitura",IF(I16&lt;$H$8,"Mais fina: investigar (polimento ou peça substituída)",IF(I16&lt;=$H$5,"Compatível",IF(I16&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo")))))</f>
         <v/>
       </c>
       <c r="L16" s="11" t="n"/>
@@ -1759,7 +1796,7 @@
         <v/>
       </c>
       <c r="K17" s="26">
-        <f>IF(B17="Plástico","NÃO MEDIR (plástico)",IF(I17="","— sem leitura",IF(I17&lt;=$H$5,"Compatível",IF(I17&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo"))))</f>
+        <f>IF(B17="Plástico","NÃO MEDIR (plástico)",IF(I17="","— sem leitura",IF(I17&lt;$H$8,"Mais fina: investigar (polimento ou peça substituída)",IF(I17&lt;=$H$5,"Compatível",IF(I17&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo")))))</f>
         <v/>
       </c>
       <c r="L17" s="11" t="n"/>
@@ -1803,7 +1840,7 @@
         <v/>
       </c>
       <c r="K18" s="26">
-        <f>IF(B18="Plástico","NÃO MEDIR (plástico)",IF(I18="","— sem leitura",IF(I18&lt;=$H$5,"Compatível",IF(I18&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo"))))</f>
+        <f>IF(B18="Plástico","NÃO MEDIR (plástico)",IF(I18="","— sem leitura",IF(I18&lt;$H$8,"Mais fina: investigar (polimento ou peça substituída)",IF(I18&lt;=$H$5,"Compatível",IF(I18&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo")))))</f>
         <v/>
       </c>
       <c r="L18" s="11" t="inlineStr">
@@ -1851,7 +1888,7 @@
         <v/>
       </c>
       <c r="K19" s="26">
-        <f>IF(B19="Plástico","NÃO MEDIR (plástico)",IF(I19="","— sem leitura",IF(I19&lt;=$H$5,"Compatível",IF(I19&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo"))))</f>
+        <f>IF(B19="Plástico","NÃO MEDIR (plástico)",IF(I19="","— sem leitura",IF(I19&lt;$H$8,"Mais fina: investigar (polimento ou peça substituída)",IF(I19&lt;=$H$5,"Compatível",IF(I19&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo")))))</f>
         <v/>
       </c>
       <c r="L19" s="11" t="n"/>
@@ -1895,7 +1932,7 @@
         <v/>
       </c>
       <c r="K20" s="26">
-        <f>IF(B20="Plástico","NÃO MEDIR (plástico)",IF(I20="","— sem leitura",IF(I20&lt;=$H$5,"Compatível",IF(I20&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo"))))</f>
+        <f>IF(B20="Plástico","NÃO MEDIR (plástico)",IF(I20="","— sem leitura",IF(I20&lt;$H$8,"Mais fina: investigar (polimento ou peça substituída)",IF(I20&lt;=$H$5,"Compatível",IF(I20&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo")))))</f>
         <v/>
       </c>
       <c r="L20" s="11" t="inlineStr">
@@ -1939,7 +1976,7 @@
         <v/>
       </c>
       <c r="K21" s="26">
-        <f>IF(B21="Plástico","NÃO MEDIR (plástico)",IF(I21="","— sem leitura",IF(I21&lt;=$H$5,"Compatível",IF(I21&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo"))))</f>
+        <f>IF(B21="Plástico","NÃO MEDIR (plástico)",IF(I21="","— sem leitura",IF(I21&lt;$H$8,"Mais fina: investigar (polimento ou peça substituída)",IF(I21&lt;=$H$5,"Compatível",IF(I21&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo")))))</f>
         <v/>
       </c>
       <c r="L21" s="11" t="n"/>
@@ -1979,7 +2016,7 @@
         <v/>
       </c>
       <c r="K22" s="26">
-        <f>IF(B22="Plástico","NÃO MEDIR (plástico)",IF(I22="","— sem leitura",IF(I22&lt;=$H$5,"Compatível",IF(I22&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo"))))</f>
+        <f>IF(B22="Plástico","NÃO MEDIR (plástico)",IF(I22="","— sem leitura",IF(I22&lt;$H$8,"Mais fina: investigar (polimento ou peça substituída)",IF(I22&lt;=$H$5,"Compatível",IF(I22&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo")))))</f>
         <v/>
       </c>
       <c r="L22" s="11" t="n"/>
@@ -1995,11 +2032,21 @@
           <t>Aço</t>
         </is>
       </c>
-      <c r="C23" s="24" t="n"/>
-      <c r="D23" s="24" t="n"/>
-      <c r="E23" s="24" t="n"/>
-      <c r="F23" s="24" t="n"/>
-      <c r="G23" s="24" t="n"/>
+      <c r="C23" s="24" t="n">
+        <v>66</v>
+      </c>
+      <c r="D23" s="24" t="n">
+        <v>68</v>
+      </c>
+      <c r="E23" s="24" t="n">
+        <v>64</v>
+      </c>
+      <c r="F23" s="24" t="n">
+        <v>67</v>
+      </c>
+      <c r="G23" s="24" t="n">
+        <v>65</v>
+      </c>
       <c r="H23" s="21">
         <f>IF(OR(B23="Plástico",COUNT(C23:G23)=0),"",AVERAGE(C23:G23))</f>
         <v/>
@@ -2013,10 +2060,14 @@
         <v/>
       </c>
       <c r="K23" s="26">
-        <f>IF(B23="Plástico","NÃO MEDIR (plástico)",IF(I23="","— sem leitura",IF(I23&lt;=$H$5,"Compatível",IF(I23&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo"))))</f>
-        <v/>
-      </c>
-      <c r="L23" s="11" t="n"/>
+        <f>IF(B23="Plástico","NÃO MEDIR (plástico)",IF(I23="","— sem leitura",IF(I23&lt;$H$8,"Mais fina: investigar (polimento ou peça substituída)",IF(I23&lt;=$H$5,"Compatível",IF(I23&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo")))))</f>
+        <v/>
+      </c>
+      <c r="L23" s="11" t="inlineStr">
+        <is>
+          <t>Exemplo: película mais fina</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="28" t="inlineStr">
@@ -2047,7 +2098,7 @@
         <v/>
       </c>
       <c r="K24" s="26">
-        <f>IF(B24="Plástico","NÃO MEDIR (plástico)",IF(I24="","— sem leitura",IF(I24&lt;=$H$5,"Compatível",IF(I24&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo"))))</f>
+        <f>IF(B24="Plástico","NÃO MEDIR (plástico)",IF(I24="","— sem leitura",IF(I24&lt;$H$8,"Mais fina: investigar (polimento ou peça substituída)",IF(I24&lt;=$H$5,"Compatível",IF(I24&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo")))))</f>
         <v/>
       </c>
       <c r="L24" s="11" t="n"/>
@@ -2081,7 +2132,7 @@
         <v/>
       </c>
       <c r="K25" s="26">
-        <f>IF(B25="Plástico","NÃO MEDIR (plástico)",IF(I25="","— sem leitura",IF(I25&lt;=$H$5,"Compatível",IF(I25&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo"))))</f>
+        <f>IF(B25="Plástico","NÃO MEDIR (plástico)",IF(I25="","— sem leitura",IF(I25&lt;$H$8,"Mais fina: investigar (polimento ou peça substituída)",IF(I25&lt;=$H$5,"Compatível",IF(I25&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo")))))</f>
         <v/>
       </c>
       <c r="L25" s="11" t="n"/>
@@ -2115,7 +2166,7 @@
         <v/>
       </c>
       <c r="K26" s="26">
-        <f>IF(B26="Plástico","NÃO MEDIR (plástico)",IF(I26="","— sem leitura",IF(I26&lt;=$H$5,"Compatível",IF(I26&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo"))))</f>
+        <f>IF(B26="Plástico","NÃO MEDIR (plástico)",IF(I26="","— sem leitura",IF(I26&lt;$H$8,"Mais fina: investigar (polimento ou peça substituída)",IF(I26&lt;=$H$5,"Compatível",IF(I26&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo")))))</f>
         <v/>
       </c>
       <c r="L26" s="11" t="n"/>
@@ -2149,7 +2200,7 @@
         <v/>
       </c>
       <c r="K27" s="26">
-        <f>IF(B27="Plástico","NÃO MEDIR (plástico)",IF(I27="","— sem leitura",IF(I27&lt;=$H$5,"Compatível",IF(I27&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo"))))</f>
+        <f>IF(B27="Plástico","NÃO MEDIR (plástico)",IF(I27="","— sem leitura",IF(I27&lt;$H$8,"Mais fina: investigar (polimento ou peça substituída)",IF(I27&lt;=$H$5,"Compatível",IF(I27&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo")))))</f>
         <v/>
       </c>
       <c r="L27" s="11" t="inlineStr">
@@ -2187,7 +2238,7 @@
         <v/>
       </c>
       <c r="K28" s="26">
-        <f>IF(B28="Plástico","NÃO MEDIR (plástico)",IF(I28="","— sem leitura",IF(I28&lt;=$H$5,"Compatível",IF(I28&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo"))))</f>
+        <f>IF(B28="Plástico","NÃO MEDIR (plástico)",IF(I28="","— sem leitura",IF(I28&lt;$H$8,"Mais fina: investigar (polimento ou peça substituída)",IF(I28&lt;=$H$5,"Compatível",IF(I28&lt;=$H$6,"Provável repintura","Provável repintura c/ massa/reparo")))))</f>
         <v/>
       </c>
       <c r="L28" s="11" t="inlineStr">
@@ -2211,78 +2262,91 @@
     <row r="31">
       <c r="A31" s="32" t="inlineStr">
         <is>
-          <t>Compatível</t>
+          <t>Mais fina: investigar</t>
         </is>
       </c>
       <c r="B31" s="33">
-        <f>COUNTIF(K10:K28,"Compatível")</f>
+        <f>COUNTIF(K10:K28,"Mais fina*")</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="32" t="inlineStr">
         <is>
-          <t>Provável repintura</t>
+          <t>Compatível</t>
         </is>
       </c>
       <c r="B32" s="33">
-        <f>COUNTIF(K10:K28,"Provável repintura")</f>
+        <f>COUNTIF(K10:K28,"Compatível")</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="32" t="inlineStr">
         <is>
-          <t>Provável repintura c/ massa/reparo</t>
+          <t>Provável repintura</t>
         </is>
       </c>
       <c r="B33" s="33">
-        <f>COUNTIF(K10:K28,"Provável repintura c/*")</f>
+        <f>COUNTIF(K10:K28,"Provável repintura")</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="32" t="inlineStr">
         <is>
-          <t>Sem leitura (metálicas)</t>
+          <t>Provável repintura c/ massa/reparo</t>
         </is>
       </c>
       <c r="B34" s="33">
-        <f>COUNTIF(K10:K28,"— sem leitura")</f>
+        <f>COUNTIF(K10:K28,"Provável repintura c/*")</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="32" t="inlineStr">
         <is>
+          <t>Sem leitura (metálicas)</t>
+        </is>
+      </c>
+      <c r="B35" s="33">
+        <f>COUNTIF(K10:K28,"— sem leitura")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="32" t="inlineStr">
+        <is>
           <t>Não medir (plástico)</t>
         </is>
       </c>
-      <c r="B35" s="33">
+      <c r="B36" s="33">
         <f>COUNTIF(K10:K28,"NÃO MEDIR*")</f>
         <v/>
       </c>
     </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="34" t="inlineStr">
-        <is>
-          <t>Valores ORIENTATIVOS: a espessura original varia por fabricante, modelo, ano, cor e processo. Limites de razão (1,3 e 2,0) são ponto de partida editável. Medidor Fe/NFe: aço no modo Fe; alumínio exige modo/sonda NFe; plástico e fibra não são medidos por esse método. Espessura alta é INDÍCIO: confirme com inspeção visual (textura, tonalidade, respingos, vedações, parafusos) antes de atribuir o nível no Registro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="30" customHeight="1"/>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="34" t="inlineStr">
+        <is>
+          <t>Valores ORIENTATIVOS: a espessura original varia por fabricante, modelo, ano, cor e processo. Limites de razão (0,7; 1,3 e 2,0) são ponto de partida editável. Razão abaixo de 0,7 (película mais fina que a referência) também é indício: investigar polimento excessivo ou peça substituída. Medidor Fe/NFe: aço no modo Fe; alumínio exige modo/sonda NFe; plástico e fibra não são medidos por esse método. Espessura alta é INDÍCIO: confirme com inspeção visual (textura, tonalidade, respingos, vedações, parafusos) antes de atribuir o nível no Registro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1"/>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="16">
     <mergeCell ref="E4:F4"/>
-    <mergeCell ref="A37:L38"/>
     <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="I8:L8"/>
     <mergeCell ref="E5:G5"/>
     <mergeCell ref="I7:J7"/>
+    <mergeCell ref="B6:D6"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="K2:L3"/>
+    <mergeCell ref="E8:G8"/>
     <mergeCell ref="G4:I4"/>
+    <mergeCell ref="A38:L39"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="E7:G7"/>
@@ -2290,24 +2354,30 @@
   </mergeCells>
   <conditionalFormatting sqref="K10:K28">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+      <formula>LEFT(K10,9)="Mais fina"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1" stopIfTrue="1">
       <formula>LEFT(K10,10)="Compatível"</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1" stopIfTrue="1">
+    <cfRule type="expression" priority="3" dxfId="2" stopIfTrue="1">
       <formula>LEFT(K10,21)="Provável repintura c/"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="2" stopIfTrue="1">
+    <cfRule type="expression" priority="4" dxfId="3" stopIfTrue="1">
       <formula>LEFT(K10,18)="Provável repintura"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="3" stopIfTrue="1">
+    <cfRule type="expression" priority="5" dxfId="4" stopIfTrue="1">
       <formula>LEFT(K10,9)="NÃO MEDIR"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I10:I28">
-    <cfRule type="expression" priority="5" dxfId="4">
+    <cfRule type="expression" priority="6" dxfId="5">
       <formula>AND(ISNUMBER(I10),I10&gt;$H$6)</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="5">
+    <cfRule type="expression" priority="7" dxfId="6">
       <formula>AND(ISNUMBER(I10),I10&gt;$H$5)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="7">
+      <formula>AND(ISNUMBER(I10),I10&lt;$H$8)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">

</xml_diff>